<commit_message>
Add direct abstract fetchers
</commit_message>
<xml_diff>
--- a/data/paper_database.xlsx
+++ b/data/paper_database.xlsx
@@ -592,7 +592,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/tmi.2026.3665561</t>
+          <t>https://ieeexplore.ieee.org/document/11397739/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Automated chest X-ray report generation requires not only clinical accuracy but also transparent and interpretable diagnostic reasoning. In this work, we propose FiR-Rad , a two-stage framework that combines explicit structured reasoning with targeted fine-grained optimization. In the first stage, a supervised chain-of-thought approach guides the model to sequentially analyze and describe a comprehensive range of clinically significant thoracic abnormalities, ensuring clinically meaningful coverage. In the second stage, we introduce a segment-level reinforcement learning strategy based on Group Relative Policy Optimization (GRPO), which assigns precise rewards to each disease-specific reasoning step by evaluating the accuracy of corresponding findings in the synthesized report. This design provides direct feedback for intermediate reasoning and encourages consistency between detailed abnormality analysis and final diagnostic conclusions. Experimental results on the MIMIC-CXR and IU-Xray datasets demonstrate that our framework achieves state-of-the-art performance across clinical and linguistic metrics, with strong zero-shot generalization on IU-Xray. The proposed method significantly enhances interpretability and clinical accuracy, effectively addressing key limitations in automated radiology report generation.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -649,10 +654,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41467-026-72776-z</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>https://www.nature.com/articles/s41467-026-72776-z</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>MRI is the most effective method for screening high-risk breast cancer patients. While current exams rely on the qualitative evaluation of morphological features before and after contrast administration and less on contrast kinetic information, recent developments in fast acquisition methods aim to combine both. However, balancing spatial resolution, temporal resolution and scan time poses a considerable challenge in dynamic MRI. Here, we introduce a radial MRI reconstruction framework for Dynamic Contrast Enhanced (DCE) imaging, termed Enhanced Locally low-rank Imaging for Tissue contrast Enhancement (ELITE), to address these limitations. ELITE combines locally low-rank subspace modeling to capture spatially localized tissue dynamics with deep learning. We evaluate its effectiveness using the publicly available fastMRI breast initiative, demonstrating substantial improvements in CNR and noise reduction while enabling flexible temporal resolution down to 1 second. ELITE also shows benefits in neck and brain imaging, making it a viable alternative for other DCE-MRI applications.</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Crossref</t>
@@ -893,10 +902,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/tmi.2026.3700856</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>https://ieeexplore.ieee.org/document/11552880/</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Chest X-Ray Vision-Language pretraining (VLP) leverages large-scale radiograph-report pairs to develop joint image-text representations, demonstrating significant potential for medical image diagnosis. However, existing VLP approaches often overlook the multi-view nature of chest X-Rays, and some multi-view methods apply uniform feature fusion, neglecting view-key semantic contributions. Moreover, random cross-modal Masked Language Modeling (MLM) fails to facilitate effective interactions, impeding representation alignment. Additionally, global alignment in VLP may lead to the false-negative problem. To address these limitations, we propose a novel medical VLP framework comprising three core components. First, a Key Semantics-enhanced Multi-view MLM module aggregates pathology-relevant patches across views, providing semantically rich supervision for MLM. A local semantics enhancing approach, which identifies and aggregates pathology-relevant key patches across views to guide MLM. Second, a Frontal-Lateral Alignment module extracts view-specific pathological features, ensuring semantic consistency and preserving critical information during aggregation. This module independently extracts pathological features from both views to preserve view-specific information while ensuring semantic consistency, which mitigates the loss of crucial information during aggregation. Third, a High-order Semantic Alignment approach mitigates false-negative issues by aligning features with semantically consistent clusters, enhancing global alignment through prototype-level semantics. Extensive experiments across seven public datasets demonstrate that our framework outperforms state-of-the-art methods in four downstream tasks, validating its efficacy. The code is available at https://github.com/sajiutea/F-L.</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Crossref</t>

</xml_diff>

<commit_message>
Add PubMed abstract fallback
</commit_message>
<xml_diff>
--- a/data/paper_database.xlsx
+++ b/data/paper_database.xlsx
@@ -535,7 +535,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.media.2026.104001</t>
+          <t>https://linkinghub.elsevier.com/retrieve/pii/S1361841526000708</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Vertebral Compression Fractures (VCFs) are early signs of osteoporosis and the most common type of osteoporotic fracture. In clinical practice, the pipeline of VCFs diagnosis consists of two examinations while most only routinely perform the first examination when the absence of clinical manifestations, leading to an underdiagnosis. In this study, we aim to explore the potential of VCFs screening in initial frontal Chest X-rays (CXRs) examination, which is more challenging for radiologists due to difficulties such as organ occlusion and inter-class similarity. We develop a two-stage framework: in the first stage, a segmentation framework and a post-processing algorithm are proposed to obtain individual vertebrae; in the second stage, the TADC-Net is proposed to perform accurate recognition of VCFs by designing a Triplet Aggregation module for contextual feature extraction and aggregation, and a Dual Contrastive Loss module for overcome inter-class similarity. Experiments conducted on three datasets collected from multi-center hospitals demonstrate that the proposed method outperforms existing approaches quantitatively and qualitatively. Moreover, a comparative analysis with two radiologists demonstrates that the proposed method exhibits optimal performance while effectively enhances radiologists' accuracy and sensitive in VCFs screening on CXRs by helping them identify additional fracture cases, verifying the potential of early screening.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">

</xml_diff>